<commit_message>
implementation of meaning-retrieving function
</commit_message>
<xml_diff>
--- a/meaning-teller.xlsx
+++ b/meaning-teller.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20379"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE292677-A7B5-40D4-98F0-B7CF8E2D77A9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BEEB376-1EF6-4E4F-ADD8-CC053A0C64D0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="9552" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,26 +20,56 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+  <si>
+    <t>greet, greeting</t>
+  </si>
   <si>
     <t>Hello</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>tank</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>q</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>s</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>x</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>used when meeting or greeting someone:</t>
-  </si>
-  <si>
-    <t>greet, greeting</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>error</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mistake</t>
+    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>https://dictionary.cambridge.org/dictionary/english/hello</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://dictionary.cambridge.org/dictionary/english/error</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts/>
-  <fonts>
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -54,8 +84,16 @@
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Yu Gothic"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills>
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -63,7 +101,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders>
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -72,13 +110,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs>
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -357,32 +398,64 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr/>
+  <dimension ref="A2:D4"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="2" max="2" width="37.296875" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="49" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B3" t="s">
         <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{86BFBFBA-3735-481C-8F73-D9907017953C}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{90275463-3AE5-43CC-92A5-68D5A6902971}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
implementation of data saving function
</commit_message>
<xml_diff>
--- a/meaning-teller.xlsx
+++ b/meaning-teller.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20379"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BEEB376-1EF6-4E4F-ADD8-CC053A0C64D0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC98A8C6-80E7-4266-914A-E2930A73BF2D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="9552" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="9552" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,56 +20,135 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>greet, greeting</t>
   </si>
   <si>
+    <t>https://dictionary.cambridge.org/dictionary/english/hello</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
     <t>Hello</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
+    <t>pail</t>
+  </si>
+  <si>
+    <t>aerosol, bottle, cansiter</t>
+  </si>
+  <si>
+    <t>https://dictionary.cambridge.org/dictionary/english/pail</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>segregate</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://dictionary.cambridge.org/dictionary/english/segregate</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>isolate, separate</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>used when meeting or greeting someone:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>to keep one thing separate from another:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>swap</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>to exchange</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>exchange</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://dictionary.cambridge.org/dictionary/english/swap</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>gain</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>to get</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>get, receive</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://dictionary.cambridge.org/dictionary/english/gain</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>provide</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>to give</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>give</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://dictionary.cambridge.org/dictionary/english/provide</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>a bucket</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>game</t>
+  </si>
+  <si>
+    <t>an entertaining activity or sport, especially one played by children, or the equipment needed for such an activity:</t>
+  </si>
+  <si>
     <t>tank</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>q</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>s</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>x</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>used when meeting or greeting someone:</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>error</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>mistake</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://dictionary.cambridge.org/dictionary/english/hello</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>https://dictionary.cambridge.org/dictionary/english/error</t>
-    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://dictionary.cambridge.org/dictionary/english/game</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">unbearable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">too painful or unpleasant for you to continue to experience:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">painful, sensitive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;https://dictionary.cambridge.org/dictionary/english/unbearable&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;https://www.merriam-webster.com/dictionary/unbearable&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <numFmts/>
+  <fonts>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -92,8 +171,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1D2A57"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills>
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -101,7 +194,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders>
     <border>
       <left/>
       <right/>
@@ -114,9 +207,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
@@ -398,7 +493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:D4"/>
+  <sheetPr/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
@@ -407,55 +502,130 @@
     <col min="4" max="4" width="49" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s" s="1">
+        <v>1</v>
+      </c>
+    </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
         <v>6</v>
       </c>
+      <c r="B2" t="s" s="2">
+        <v>10</v>
+      </c>
       <c r="C2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="D2" t="s" s="1">
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="1">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="B4" t="s" s="3">
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
+      </c>
+      <c r="D4" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s" s="3">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s" s="1">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" t="s" s="3">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" t="s" s="1">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <hyperlinks>
-    <hyperlink ref="D4" r:id="rId1" xr:uid="{86BFBFBA-3735-481C-8F73-D9907017953C}"/>
-    <hyperlink ref="D2" r:id="rId2" xr:uid="{90275463-3AE5-43CC-92A5-68D5A6902971}"/>
+    <hyperlink ref="D1" r:id="rId1" xr:uid="{D2457F67-1A79-4D39-B96B-4FE27E2293A4}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{295A93DA-F2A7-4E4E-89F3-FE83B9BA2BEB}"/>
+    <hyperlink ref="D3" r:id="rId3" xr:uid="{32A75493-035A-4B7E-AA44-B565CEBAB3CC}"/>
+    <hyperlink ref="D4" r:id="rId4" xr:uid="{C3F8116F-D05C-469F-B7C6-052E2B7C700F}"/>
+    <hyperlink ref="D5" r:id="rId5" xr:uid="{3CBC0BEF-7670-4E8C-BB1D-D1E9C94CC243}"/>
+    <hyperlink ref="D6" r:id="rId6" xr:uid="{114457BA-E27F-43E7-AD8D-21AC564C75CE}"/>
+    <hyperlink ref="D7" r:id="rId7" xr:uid="{8ED0E385-BD94-4088-82BA-824551E8487C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix error of auto-generating function in case of there is no exactly mathced word.[D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[1;2D[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[C[D[D[D[D[D[D[D[D[D[D[D[D[D[D[D[D[D[C[C[C[C[C[C[D[D[D[D when excute ""[Dtamea ()[Dword[C"[D[D)
</commit_message>
<xml_diff>
--- a/meaning-teller.xlsx
+++ b/meaning-teller.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20379"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5692B920-4570-4B8C-9A1D-8B18561FE191}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CADBD99C-E461-4DD4-A0C0-FDB84625F8B1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="9552" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="9552" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>greet, greeting</t>
   </si>
@@ -149,15 +149,74 @@
     <t>https://dictionary.cambridge.org/dictionary/english/fire</t>
   </si>
   <si>
+    <t>rifle</t>
+  </si>
+  <si>
+    <t>search and rob, plunder, go through, pillage</t>
+  </si>
+  <si>
+    <t>https://dictionary.cambridge.org/dictionary/english/rifle</t>
+  </si>
+  <si>
+    <t>direct</t>
+  </si>
+  <si>
+    <t>supervise, oversee, head, serve as director for</t>
+  </si>
+  <si>
+    <t>https://dictionary.cambridge.org/dictionary/english/direct</t>
+  </si>
+  <si>
     <t>tank</t>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>message</t>
+  </si>
+  <si>
+    <t>notice, word, statement, news</t>
+  </si>
+  <si>
+    <t>https://dictionary.cambridge.org/dictionary/english/message</t>
+  </si>
+  <si>
+    <t>a &lt;https://dictionary.cambridge.org/dictionary/english/short|short&gt; &lt;https://dictionary.cambridge.org/dictionary/english/piece|piece&gt; of &lt;https://dictionary.cambridge.org/dictionary/english/information|information&gt; that you give to a &lt;https://dictionary.cambridge.org/dictionary/english/person|person&gt; when you cannot &lt;https://dictionary.cambridge.org/dictionary/english/speak|speak&gt; to them &lt;https://dictionary.cambridge.org/dictionary/english/directly|directly&gt;:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">update</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tell, give, communicate, inform</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://dictionary.cambridge.org/dictionary/english/update</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to make something more modern</t>
+  </si>
+  <si>
+    <t xml:space="preserve">synonym</t>
+  </si>
+  <si>
+    <t xml:space="preserve">equivalent word, analogue, equivalent, another name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://dictionary.cambridge.org/dictionary/english/synonym</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a word or phrase that has the same or nearly the same meaning</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <numFmts/>
+  <fonts>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -195,7 +254,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills>
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -203,7 +262,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders>
     <border>
       <left/>
       <right/>
@@ -216,7 +275,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -502,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D9"/>
+  <sheetPr/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
@@ -521,7 +580,7 @@
       <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s" s="1">
         <v>1</v>
       </c>
     </row>
@@ -529,13 +588,13 @@
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s" s="2">
         <v>10</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s" s="1">
         <v>7</v>
       </c>
     </row>
@@ -549,7 +608,7 @@
       <c r="C3" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s" s="1">
         <v>5</v>
       </c>
     </row>
@@ -557,13 +616,13 @@
       <c r="A4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" t="s" s="3">
         <v>12</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" t="s" s="1">
         <v>14</v>
       </c>
     </row>
@@ -571,13 +630,13 @@
       <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" t="s" s="3">
         <v>16</v>
       </c>
       <c r="C5" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" t="s" s="1">
         <v>18</v>
       </c>
     </row>
@@ -585,13 +644,13 @@
       <c r="A6" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" t="s" s="3">
         <v>20</v>
       </c>
       <c r="C6" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s" s="1">
         <v>22</v>
       </c>
     </row>
@@ -605,7 +664,7 @@
       <c r="C7" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" t="s" s="1">
         <v>26</v>
       </c>
     </row>
@@ -628,13 +687,83 @@
         <v>32</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
         <v>33</v>
       </c>
       <c r="D9" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>